<commit_message>
data: actualiser le recensement Mosar (nicocoquet)
</commit_message>
<xml_diff>
--- a/data/Recensement-revues-Mosar.xlsx
+++ b/data/Recensement-revues-Mosar.xlsx
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -784,6 +784,7 @@
           <t>parution continue</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -943,10 +944,10 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -1091,6 +1092,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1323,6 +1325,7 @@
           <t>Bulletin de la Société préhistorique française</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>BSPF</t>
@@ -1350,10 +1353,10 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1401,6 +1404,7 @@
       <c r="W5" t="n">
         <v>4</v>
       </c>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -1496,11 +1500,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT5" t="inlineStr"/>
       <c r="AU5" t="inlineStr">
         <is>
           <t>0</t>
@@ -1928,6 +1934,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1950,6 +1957,7 @@
           <t>Espaces et sociétés</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>0014-0481</t>
@@ -1972,10 +1980,10 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -2078,6 +2086,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr">
         <is>
           <t>0</t>
@@ -2088,11 +2097,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr">
         <is>
           <t>1</t>
@@ -2150,6 +2161,7 @@
           <t>Ethnologie française</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>0046-2616</t>
@@ -2172,10 +2184,10 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -2328,6 +2340,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2350,6 +2363,7 @@
           <t>Études Lawrenciennes</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>0994-5490</t>
@@ -2599,10 +2613,10 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -2632,6 +2646,7 @@
       <c r="S11" t="n">
         <v>1960</v>
       </c>
+      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
           <t>1960's</t>
@@ -2645,6 +2660,7 @@
       <c r="W11" t="n">
         <v>3</v>
       </c>
+      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -2725,16 +2741,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT11" t="inlineStr"/>
       <c r="AU11" t="inlineStr">
         <is>
           <t>0</t>
@@ -2809,10 +2828,10 @@
         <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -2915,6 +2934,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL12" t="inlineStr"/>
       <c r="AM12" t="inlineStr">
         <is>
           <t>0</t>
@@ -2925,6 +2945,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr">
         <is>
           <t>1</t>
@@ -2940,6 +2961,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT12" t="inlineStr"/>
       <c r="AU12" t="inlineStr">
         <is>
           <t>1</t>
@@ -3024,10 +3046,10 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3160,6 +3182,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr">
         <is>
           <t>1</t>
@@ -3175,6 +3198,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT13" t="inlineStr"/>
       <c r="AU13" t="inlineStr">
         <is>
           <t>1</t>
@@ -3232,6 +3256,7 @@
           <t>Journal de la Société des américanistes</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>JSA</t>
@@ -3259,10 +3284,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -3292,6 +3317,7 @@
       <c r="S14" t="n">
         <v>1895</v>
       </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
           <t>XIXe siècle</t>
@@ -3305,6 +3331,7 @@
       <c r="W14" t="n">
         <v>2</v>
       </c>
+      <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -3370,6 +3397,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="inlineStr">
         <is>
           <t>1</t>
@@ -3385,6 +3413,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr">
         <is>
           <t>1</t>
@@ -3400,6 +3429,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT14" t="inlineStr"/>
       <c r="AU14" t="inlineStr">
         <is>
           <t>1</t>
@@ -3457,6 +3487,7 @@
           <t>Justice spatiale/Spatial Justice</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>jssj</t>
@@ -3482,7 +3513,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -3512,6 +3543,7 @@
       <c r="S15" t="n">
         <v>2009</v>
       </c>
+      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
           <t>2000's</t>
@@ -3525,6 +3557,7 @@
       <c r="W15" t="n">
         <v>1</v>
       </c>
+      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -3625,6 +3658,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3647,6 +3681,7 @@
           <t>L'Atelier</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>2109-9103</t>
@@ -3815,6 +3850,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4057,6 +4093,7 @@
           <t>Littérales</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>2802-3293</t>
@@ -4267,6 +4304,7 @@
           <t>Matériaux pour l'histoire de notre temps</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>0769-3206</t>
@@ -4400,6 +4438,7 @@
           <t>pas de mention = Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL19" t="inlineStr"/>
       <c r="AM19" t="inlineStr">
         <is>
           <t>0</t>
@@ -4410,11 +4449,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP19" t="inlineStr"/>
       <c r="AQ19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr">
         <is>
           <t>1</t>
@@ -4660,6 +4701,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4709,10 +4751,10 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -4897,6 +4939,7 @@
           <t>Photographica</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>2780-8572</t>
@@ -5025,6 +5068,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL22" t="inlineStr"/>
       <c r="AM22" t="inlineStr">
         <is>
           <t>0</t>
@@ -5035,6 +5079,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="inlineStr">
         <is>
           <t>1</t>
@@ -5050,6 +5095,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT22" t="inlineStr"/>
       <c r="AU22" t="inlineStr">
         <is>
           <t>1</t>
@@ -5107,6 +5153,7 @@
           <t>Revue d'histoire des sciences humaines</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>RHSH</t>
@@ -5167,6 +5214,7 @@
       <c r="S23" t="n">
         <v>1999</v>
       </c>
+      <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr">
         <is>
           <t>1990's</t>
@@ -5180,6 +5228,7 @@
       <c r="W23" t="n">
         <v>2</v>
       </c>
+      <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -5240,6 +5289,7 @@
           <t>CC BY</t>
         </is>
       </c>
+      <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr">
         <is>
           <t>0</t>
@@ -5250,6 +5300,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr">
         <is>
           <t>1</t>
@@ -5327,6 +5378,7 @@
           <t>Revue internationale des études du développement</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>Ried</t>
@@ -5405,6 +5457,7 @@
       <c r="W24" t="n">
         <v>3</v>
       </c>
+      <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -5520,6 +5573,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5542,6 +5596,7 @@
           <t>Sociétés &amp; Représentations</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>1262-2966</t>
@@ -5747,6 +5802,7 @@
           <t>Socio-anthropologie</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>1276-8707</t>
@@ -5984,10 +6040,10 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -6172,6 +6228,7 @@
           <t>Terrains/Théories</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>2427-9188</t>
@@ -6409,10 +6466,10 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -6597,6 +6654,7 @@
           <t>Actuel Marx</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>0994-4524</t>
@@ -6935,6 +6993,7 @@
           <t>CC BY-NC</t>
         </is>
       </c>
+      <c r="AL31" t="inlineStr"/>
       <c r="AM31" t="inlineStr">
         <is>
           <t>0</t>
@@ -6945,6 +7004,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP31" t="inlineStr"/>
       <c r="AQ31" t="inlineStr">
         <is>
           <t>1</t>
@@ -6960,6 +7020,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT31" t="inlineStr"/>
       <c r="AU31" t="inlineStr">
         <is>
           <t>1</t>
@@ -7227,6 +7288,7 @@
           <t>Approches Théoriques en Information-Communication</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>ATIC</t>
@@ -7405,6 +7467,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7427,6 +7490,7 @@
           <t>Archives de politique criminelle</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>0242-5637</t>
@@ -7555,6 +7619,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL34" t="inlineStr"/>
       <c r="AM34" t="inlineStr">
         <is>
           <t>0</t>
@@ -7565,11 +7630,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP34" t="inlineStr"/>
       <c r="AQ34" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR34" t="inlineStr"/>
       <c r="AS34" t="inlineStr">
         <is>
           <t>1</t>
@@ -7797,6 +7864,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7997,6 +8065,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8172,11 +8241,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP37" t="inlineStr"/>
       <c r="AQ37" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR37" t="inlineStr"/>
       <c r="AS37" t="inlineStr">
         <is>
           <t>1</t>
@@ -8234,6 +8305,7 @@
           <t>Cahiers du Centre Gustave-Glotz</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>1016-9008</t>
@@ -8392,11 +8464,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR38" t="inlineStr"/>
       <c r="AS38" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT38" t="inlineStr"/>
       <c r="AU38" t="inlineStr">
         <is>
           <t>0</t>
@@ -8654,6 +8728,7 @@
           <t>Crisol</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>0764-7611</t>
@@ -8829,6 +8904,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9063,6 +9139,7 @@
           <t>Design, Arts, Médias</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>2743-0332</t>
@@ -9228,6 +9305,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9250,6 +9328,7 @@
           <t>Documents de travail du Centre d'économie de la Sorbonne</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>DT du CES</t>
@@ -9330,6 +9409,7 @@
           <t>irrégulier</t>
         </is>
       </c>
+      <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -9430,6 +9510,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9452,6 +9533,7 @@
           <t>EchoGéo</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>1963-1197</t>
@@ -9825,6 +9907,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10047,6 +10130,7 @@
           <t>L'Espace géographique</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>0046-2497</t>
@@ -10175,6 +10259,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL47" t="inlineStr"/>
       <c r="AM47" t="inlineStr">
         <is>
           <t>1</t>
@@ -10200,6 +10285,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr">
         <is>
           <t>1</t>
@@ -10317,6 +10403,7 @@
       <c r="S48" t="n">
         <v>2012</v>
       </c>
+      <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr">
         <is>
           <t>2010's</t>
@@ -10330,6 +10417,7 @@
       <c r="W48" t="n">
         <v>2</v>
       </c>
+      <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -10467,6 +10555,7 @@
           <t>Le Mouvement social</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>0027-2671</t>
@@ -10620,11 +10709,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP49" t="inlineStr"/>
       <c r="AQ49" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr">
         <is>
           <t>1</t>
@@ -10855,6 +10946,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11255,6 +11347,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11277,6 +11370,7 @@
           <t>Philonsorbonne</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>1961-4829</t>
@@ -11660,6 +11754,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12047,6 +12142,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -12069,6 +12165,7 @@
           <t>Revue d'histoire du XIXe siècle</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>1265-1354</t>
@@ -12202,6 +12299,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL57" t="inlineStr"/>
       <c r="AM57" t="inlineStr">
         <is>
           <t>0</t>
@@ -12284,6 +12382,7 @@
           <t>Revue économique</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>0035-2764</t>
@@ -12432,11 +12531,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP58" t="inlineStr"/>
       <c r="AQ58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr">
         <is>
           <t>1</t>
@@ -12494,6 +12595,7 @@
           <t>Revue internationale de l'éducation familiale</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>Rief</t>
@@ -12554,6 +12656,7 @@
       <c r="S59" t="n">
         <v>1997</v>
       </c>
+      <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr">
         <is>
           <t>1990's</t>
@@ -12567,6 +12670,7 @@
       <c r="W59" t="n">
         <v>2</v>
       </c>
+      <c r="X59" t="inlineStr"/>
       <c r="Y59" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -12642,11 +12746,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP59" t="inlineStr"/>
       <c r="AQ59" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR59" t="inlineStr"/>
       <c r="AS59" t="inlineStr">
         <is>
           <t>1</t>
@@ -12867,6 +12973,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12889,6 +12996,7 @@
           <t>Salariat</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>2967-6266</t>
@@ -13057,6 +13165,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13232,11 +13341,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP62" t="inlineStr"/>
       <c r="AQ62" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR62" t="inlineStr"/>
       <c r="AS62" t="inlineStr">
         <is>
           <t>1</t>
@@ -13354,6 +13465,7 @@
       <c r="S63" t="n">
         <v>2018</v>
       </c>
+      <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr">
         <is>
           <t>2010's</t>
@@ -13367,6 +13479,7 @@
       <c r="W63" t="n">
         <v>2</v>
       </c>
+      <c r="X63" t="inlineStr"/>
       <c r="Y63" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -13467,6 +13580,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -13627,6 +13741,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL64" t="inlineStr"/>
       <c r="AM64" t="inlineStr">
         <is>
           <t>0</t>
@@ -13637,11 +13752,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP64" t="inlineStr"/>
       <c r="AQ64" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR64" t="inlineStr"/>
       <c r="AS64" t="inlineStr">
         <is>
           <t>1</t>
@@ -13909,6 +14026,7 @@
           <t>Actes de la recherche en sciences sociales</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>ARSS</t>
@@ -13963,6 +14081,7 @@
       <c r="S66" t="n">
         <v>1975</v>
       </c>
+      <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr">
         <is>
           <t>1970's</t>
@@ -14051,11 +14170,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP66" t="inlineStr"/>
       <c r="AQ66" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR66" t="inlineStr"/>
       <c r="AS66" t="inlineStr">
         <is>
           <t>1</t>
@@ -14281,6 +14402,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -14303,6 +14425,7 @@
           <t>Analisi e diritto</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>1126-5779</t>
@@ -14460,6 +14583,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -14629,11 +14753,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP69" t="inlineStr"/>
       <c r="AQ69" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR69" t="inlineStr"/>
       <c r="AS69" t="inlineStr">
         <is>
           <t>1</t>
@@ -14691,6 +14817,7 @@
           <t>Annales de géographie</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>0003-4010</t>
@@ -14828,11 +14955,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP70" t="inlineStr"/>
       <c r="AQ70" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR70" t="inlineStr"/>
       <c r="AS70" t="inlineStr">
         <is>
           <t>1</t>
@@ -14949,6 +15078,7 @@
       <c r="S71" t="n">
         <v>1993</v>
       </c>
+      <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr">
         <is>
           <t>1990's</t>
@@ -14962,6 +15092,7 @@
       <c r="W71" t="n">
         <v>1</v>
       </c>
+      <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -15032,16 +15163,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP71" t="inlineStr"/>
       <c r="AQ71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR71" t="inlineStr"/>
       <c r="AS71" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT71" t="inlineStr"/>
       <c r="AU71" t="inlineStr">
         <is>
           <t>0</t>
@@ -15089,6 +15223,7 @@
           <t>Archéologie, société et environnement</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>2752-4507</t>
@@ -15226,6 +15361,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -15248,6 +15384,7 @@
           <t>Articulation(s)</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>2728-834X</t>
@@ -15400,6 +15537,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -16002,6 +16140,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -16024,6 +16163,7 @@
           <t>Cahiers d'études africaines</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>0008-0055</t>
@@ -16161,6 +16301,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP77" t="inlineStr"/>
       <c r="AQ77" t="inlineStr">
         <is>
           <t>1</t>
@@ -16564,6 +16705,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -16763,6 +16905,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -16785,6 +16928,7 @@
           <t>Cultures &amp; Conflits</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>1157-996X</t>
@@ -16922,6 +17066,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP81" t="inlineStr"/>
       <c r="AQ81" t="inlineStr">
         <is>
           <t>1</t>
@@ -17515,6 +17660,7 @@
           <t>CC BY-NC-ND</t>
         </is>
       </c>
+      <c r="AL84" t="inlineStr"/>
       <c r="AM84" t="inlineStr">
         <is>
           <t>0</t>
@@ -17525,6 +17671,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP84" t="inlineStr"/>
       <c r="AQ84" t="inlineStr">
         <is>
           <t>1</t>
@@ -17540,6 +17687,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT84" t="inlineStr"/>
       <c r="AU84" t="inlineStr">
         <is>
           <t>1</t>
@@ -17592,6 +17740,7 @@
           <t>Finance</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>0752-6180</t>
@@ -17709,6 +17858,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL85" t="inlineStr"/>
       <c r="AM85" t="inlineStr">
         <is>
           <t>0</t>
@@ -17719,11 +17869,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP85" t="inlineStr"/>
       <c r="AQ85" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR85" t="inlineStr"/>
       <c r="AS85" t="inlineStr">
         <is>
           <t>1</t>
@@ -17943,6 +18095,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17965,6 +18118,7 @@
           <t>French Politics</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>1476-3419</t>
@@ -18149,6 +18303,7 @@
           <t>Géographie et cultures</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>1165-0354</t>
@@ -18287,6 +18442,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP88" t="inlineStr"/>
       <c r="AQ88" t="inlineStr">
         <is>
           <t>1</t>
@@ -18302,6 +18458,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT88" t="inlineStr"/>
       <c r="AU88" t="inlineStr">
         <is>
           <t>1</t>
@@ -18521,6 +18678,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -18744,6 +18902,7 @@
           <t>International Economics</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>2110-7017</t>
@@ -18881,16 +19040,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP91" t="inlineStr"/>
       <c r="AQ91" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR91" t="inlineStr"/>
       <c r="AS91" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT91" t="inlineStr"/>
       <c r="AU91" t="inlineStr">
         <is>
           <t>0</t>
@@ -18938,6 +19100,7 @@
           <t>International Review of Social Psychology</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>IRPS</t>
@@ -19005,6 +19168,7 @@
       <c r="W92" t="n">
         <v>1</v>
       </c>
+      <c r="X92" t="inlineStr"/>
       <c r="Y92" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -19105,6 +19269,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -19127,6 +19292,7 @@
           <t>Journal d'archéologie expérimentale</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>Pas de rattachement direct à une université</t>
@@ -19153,6 +19319,26 @@
           <t>SHS</t>
         </is>
       </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
       <c r="Y93" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -19178,6 +19364,11 @@
           <t>pépinière</t>
         </is>
       </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
       <c r="AH93" t="inlineStr">
         <is>
           <t>oui</t>
@@ -19233,6 +19424,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19255,6 +19447,7 @@
           <t>Journal des africanistes</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>0399-0346</t>
@@ -19377,6 +19570,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL94" t="inlineStr"/>
       <c r="AM94" t="inlineStr">
         <is>
           <t>0</t>
@@ -19387,6 +19581,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP94" t="inlineStr"/>
       <c r="AQ94" t="inlineStr">
         <is>
           <t>1</t>
@@ -19402,6 +19597,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT94" t="inlineStr"/>
       <c r="AU94" t="inlineStr">
         <is>
           <t>0</t>
@@ -19449,6 +19645,7 @@
           <t>Journal of Archaeological Method and Theory</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>1072-5369</t>
@@ -19591,16 +19788,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP95" t="inlineStr"/>
       <c r="AQ95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR95" t="inlineStr"/>
       <c r="AS95" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT95" t="inlineStr"/>
       <c r="AU95" t="inlineStr">
         <is>
           <t>0</t>
@@ -19648,6 +19848,7 @@
           <t>Journal of Eastern African Studies</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>1753-1055</t>
@@ -19780,16 +19981,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP96" t="inlineStr"/>
       <c r="AQ96" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR96" t="inlineStr"/>
       <c r="AS96" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT96" t="inlineStr"/>
       <c r="AU96" t="inlineStr">
         <is>
           <t>0</t>
@@ -19837,6 +20041,7 @@
           <t>Journal of Islamic Manuscripts</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>1878-4631</t>
@@ -19979,6 +20184,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -20352,6 +20558,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -20511,11 +20718,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP100" t="inlineStr"/>
       <c r="AQ100" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR100" t="inlineStr"/>
       <c r="AS100" t="inlineStr">
         <is>
           <t>1</t>
@@ -20777,6 +20986,7 @@
           <t>Multitudes</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>0292-0107</t>
@@ -20909,11 +21119,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP102" t="inlineStr"/>
       <c r="AQ102" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR102" t="inlineStr"/>
       <c r="AS102" t="inlineStr">
         <is>
           <t>1</t>
@@ -21030,6 +21242,7 @@
       <c r="S103" t="n">
         <v>1993</v>
       </c>
+      <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr">
         <is>
           <t>1990's</t>
@@ -21043,6 +21256,7 @@
       <c r="W103" t="n">
         <v>4</v>
       </c>
+      <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -21113,11 +21327,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP103" t="inlineStr"/>
       <c r="AQ103" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR103" t="inlineStr"/>
       <c r="AS103" t="inlineStr">
         <is>
           <t>1</t>
@@ -21352,6 +21568,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -21374,6 +21591,7 @@
           <t>Nuevo Mundo, Mundos Nuevos</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
           <t>1626-0252</t>
@@ -21570,6 +21788,7 @@
           <t>passés futurs</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>PF</t>
@@ -21619,6 +21838,7 @@
       <c r="S106" t="n">
         <v>2017</v>
       </c>
+      <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr">
         <is>
           <t>2010's</t>
@@ -21632,6 +21852,7 @@
       <c r="W106" t="n">
         <v>2</v>
       </c>
+      <c r="X106" t="inlineStr"/>
       <c r="Y106" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -21727,6 +21948,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -21749,6 +21971,7 @@
           <t>Philosophique</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>0980-0891</t>
@@ -21871,6 +22094,7 @@
           <t>CC BY</t>
         </is>
       </c>
+      <c r="AL107" t="inlineStr"/>
       <c r="AM107" t="inlineStr">
         <is>
           <t>0</t>
@@ -21881,6 +22105,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP107" t="inlineStr"/>
       <c r="AQ107" t="inlineStr">
         <is>
           <t>1</t>
@@ -21896,6 +22121,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT107" t="inlineStr"/>
       <c r="AU107" t="inlineStr">
         <is>
           <t>1</t>
@@ -21948,6 +22174,7 @@
           <t>Politique africaine</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>0244-7827</t>
@@ -22090,6 +22317,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR108" t="inlineStr"/>
       <c r="AS108" t="inlineStr">
         <is>
           <t>1</t>
@@ -22147,6 +22375,7 @@
           <t>Politique américaine</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>1771-8848</t>
@@ -22284,11 +22513,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP109" t="inlineStr"/>
       <c r="AQ109" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR109" t="inlineStr"/>
       <c r="AS109" t="inlineStr">
         <is>
           <t>1</t>
@@ -22468,6 +22699,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL110" t="inlineStr"/>
       <c r="AM110" t="inlineStr">
         <is>
           <t>0</t>
@@ -22478,6 +22710,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP110" t="inlineStr"/>
       <c r="AQ110" t="inlineStr">
         <is>
           <t>1</t>
@@ -22493,6 +22726,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT110" t="inlineStr"/>
       <c r="AU110" t="inlineStr">
         <is>
           <t>1</t>
@@ -22692,6 +22926,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -22714,6 +22949,7 @@
           <t>Recherches familiales</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>1763-718X</t>
@@ -22846,11 +23082,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP112" t="inlineStr"/>
       <c r="AQ112" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR112" t="inlineStr"/>
       <c r="AS112" t="inlineStr">
         <is>
           <t>1</t>
@@ -23080,6 +23318,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -23301,6 +23540,7 @@
           <t>Revue d'histoire culturelle : XVIIIe-XXIe siècles</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>RHC</t>
@@ -23350,6 +23590,7 @@
       <c r="S115" t="n">
         <v>2020</v>
       </c>
+      <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr">
         <is>
           <t>2020's</t>
@@ -23505,6 +23746,7 @@
           <t>Revue d'histoire de la protection sociale</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>RHPS</t>
@@ -23577,6 +23819,7 @@
       <c r="W116" t="n">
         <v>1</v>
       </c>
+      <c r="X116" t="inlineStr"/>
       <c r="Y116" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -23632,6 +23875,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL116" t="inlineStr"/>
       <c r="AM116" t="inlineStr">
         <is>
           <t>0</t>
@@ -23642,11 +23886,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP116" t="inlineStr"/>
       <c r="AQ116" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR116" t="inlineStr"/>
       <c r="AS116" t="inlineStr">
         <is>
           <t>1</t>
@@ -23704,6 +23950,7 @@
           <t>Revue de l'arbitrage</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>0556-7440</t>
@@ -23851,6 +24098,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -23873,6 +24121,7 @@
           <t>Revue de science criminelle et de droit pénal comparé</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>RSC</t>
@@ -23933,6 +24182,7 @@
       <c r="S118" t="n">
         <v>1936</v>
       </c>
+      <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr">
         <is>
           <t>1925-1949</t>
@@ -23946,6 +24196,7 @@
       <c r="W118" t="n">
         <v>4</v>
       </c>
+      <c r="X118" t="inlineStr"/>
       <c r="Y118" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -24016,11 +24267,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP118" t="inlineStr"/>
       <c r="AQ118" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR118" t="inlineStr"/>
       <c r="AS118" t="inlineStr">
         <is>
           <t>1</t>
@@ -24078,6 +24331,7 @@
           <t>Revue des études grecques</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>REG</t>
@@ -24150,6 +24404,7 @@
       <c r="W119" t="n">
         <v>2</v>
       </c>
+      <c r="X119" t="inlineStr"/>
       <c r="Y119" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -24235,11 +24490,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR119" t="inlineStr"/>
       <c r="AS119" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT119" t="inlineStr"/>
       <c r="AU119" t="inlineStr">
         <is>
           <t>0</t>
@@ -24346,6 +24603,7 @@
       <c r="S120" t="n">
         <v>2008</v>
       </c>
+      <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr">
         <is>
           <t>2000's</t>
@@ -24359,6 +24617,7 @@
       <c r="W120" t="n">
         <v>1</v>
       </c>
+      <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -24429,16 +24688,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP120" t="inlineStr"/>
       <c r="AQ120" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR120" t="inlineStr"/>
       <c r="AS120" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT120" t="inlineStr"/>
       <c r="AU120" t="inlineStr">
         <is>
           <t>0</t>
@@ -24486,6 +24748,7 @@
           <t>Social Choice and Welfare</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>0176-1714</t>
@@ -24628,16 +24891,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP121" t="inlineStr"/>
       <c r="AQ121" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR121" t="inlineStr"/>
       <c r="AS121" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT121" t="inlineStr"/>
       <c r="AU121" t="inlineStr">
         <is>
           <t>0</t>
@@ -24828,6 +25094,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP122" t="inlineStr"/>
       <c r="AQ122" t="inlineStr">
         <is>
           <t>1</t>
@@ -24895,6 +25162,7 @@
           <t>Activités</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>1765-2723</t>
@@ -25089,6 +25357,7 @@
           <t>American Journal of Industrial and Business Management</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>2164-5167</t>
@@ -25221,16 +25490,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP124" t="inlineStr"/>
       <c r="AQ124" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR124" t="inlineStr"/>
       <c r="AS124" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT124" t="inlineStr"/>
       <c r="AU124" t="inlineStr">
         <is>
           <t>0</t>
@@ -25278,6 +25550,7 @@
           <t>Archives de philosophie</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>0003-9632</t>
@@ -25415,11 +25688,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP125" t="inlineStr"/>
       <c r="AQ125" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR125" t="inlineStr"/>
       <c r="AS125" t="inlineStr">
         <is>
           <t>1</t>
@@ -25477,6 +25752,7 @@
           <t>Brain and Cognition</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>0278-2626</t>
@@ -25609,16 +25885,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP126" t="inlineStr"/>
       <c r="AQ126" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR126" t="inlineStr"/>
       <c r="AS126" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT126" t="inlineStr"/>
       <c r="AU126" t="inlineStr">
         <is>
           <t>0</t>
@@ -25666,6 +25945,7 @@
           <t>Brain and Language</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>0093-934X</t>
@@ -25798,16 +26078,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP127" t="inlineStr"/>
       <c r="AQ127" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR127" t="inlineStr"/>
       <c r="AS127" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT127" t="inlineStr"/>
       <c r="AU127" t="inlineStr">
         <is>
           <t>0</t>
@@ -25855,6 +26138,7 @@
           <t>British journal for the history of philosophy</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>0960-8788</t>
@@ -26044,6 +26328,7 @@
           <t>Bulletin critique des annales islamologiques</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>BCAI</t>
@@ -26098,6 +26383,7 @@
       <c r="S129" t="n">
         <v>1984</v>
       </c>
+      <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr">
         <is>
           <t>1980's</t>
@@ -26111,6 +26397,7 @@
       <c r="W129" t="n">
         <v>1</v>
       </c>
+      <c r="X129" t="inlineStr"/>
       <c r="Y129" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -26181,6 +26468,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP129" t="inlineStr"/>
       <c r="AQ129" t="inlineStr">
         <is>
           <t>1</t>
@@ -26196,6 +26484,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT129" t="inlineStr"/>
       <c r="AU129" t="inlineStr">
         <is>
           <t>1</t>
@@ -26248,6 +26537,7 @@
           <t>Bulletin de l'Association de géographes français</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>BAGF</t>
@@ -26263,6 +26553,7 @@
           <t>2275-5195</t>
         </is>
       </c>
+      <c r="I130" t="inlineStr"/>
       <c r="J130" t="n">
         <v>4</v>
       </c>
@@ -26297,6 +26588,7 @@
       <c r="S130" t="n">
         <v>1924</v>
       </c>
+      <c r="T130" t="inlineStr"/>
       <c r="U130" t="inlineStr">
         <is>
           <t>1900-1924</t>
@@ -26310,6 +26602,7 @@
       <c r="W130" t="n">
         <v>4</v>
       </c>
+      <c r="X130" t="inlineStr"/>
       <c r="Y130" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -26365,6 +26658,7 @@
           <t>CC BY</t>
         </is>
       </c>
+      <c r="AL130" t="inlineStr"/>
       <c r="AM130" t="inlineStr">
         <is>
           <t>0</t>
@@ -26395,6 +26689,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT130" t="inlineStr"/>
       <c r="AU130" t="inlineStr">
         <is>
           <t>1</t>
@@ -26452,6 +26747,7 @@
           <t>Cahiers des Amériques latines</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>CAL</t>
@@ -26666,6 +26962,7 @@
           <t>Cahiers Droit, Sciences &amp; Technologies</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>Cahiers DST</t>
@@ -26720,6 +27017,7 @@
       <c r="S132" t="n">
         <v>2008</v>
       </c>
+      <c r="T132" t="inlineStr"/>
       <c r="U132" t="inlineStr">
         <is>
           <t>2000's</t>
@@ -26733,6 +27031,7 @@
       <c r="W132" t="n">
         <v>1</v>
       </c>
+      <c r="X132" t="inlineStr"/>
       <c r="Y132" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -26788,6 +27087,7 @@
           <t>CC BY</t>
         </is>
       </c>
+      <c r="AL132" t="inlineStr"/>
       <c r="AM132" t="inlineStr">
         <is>
           <t>0</t>
@@ -26798,6 +27098,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP132" t="inlineStr"/>
       <c r="AQ132" t="inlineStr">
         <is>
           <t>1</t>
@@ -26813,6 +27114,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT132" t="inlineStr"/>
       <c r="AU132" t="inlineStr">
         <is>
           <t>1</t>
@@ -26870,6 +27172,7 @@
           <t>Caravelle</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>1147-6753</t>
@@ -26992,6 +27295,7 @@
           <t>CC BY-NC-ND</t>
         </is>
       </c>
+      <c r="AL133" t="inlineStr"/>
       <c r="AM133" t="inlineStr">
         <is>
           <t>1</t>
@@ -27027,6 +27331,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT133" t="inlineStr"/>
       <c r="AU133" t="inlineStr">
         <is>
           <t>1</t>
@@ -27283,6 +27588,7 @@
           <t>Composite Structures</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
           <t>0263-8223</t>
@@ -27420,16 +27726,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP135" t="inlineStr"/>
       <c r="AQ135" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR135" t="inlineStr"/>
       <c r="AS135" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT135" t="inlineStr"/>
       <c r="AU135" t="inlineStr">
         <is>
           <t>0</t>
@@ -27477,6 +27786,7 @@
           <t>Contrats et marchés publics</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>1624-8716</t>
@@ -27634,6 +27944,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -27803,6 +28114,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -27825,6 +28137,7 @@
           <t>Economic Theory</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>0938-2259</t>
@@ -27962,16 +28275,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP138" t="inlineStr"/>
       <c r="AQ138" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR138" t="inlineStr"/>
       <c r="AS138" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT138" t="inlineStr"/>
       <c r="AU138" t="inlineStr">
         <is>
           <t>0</t>
@@ -28019,6 +28335,7 @@
           <t>Encyclopédie berbère</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>1015-7344</t>
@@ -28183,6 +28500,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -28399,6 +28717,7 @@
           <t>European Journal of English Studies</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>1382-5577</t>
@@ -28541,6 +28860,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -28563,6 +28883,7 @@
           <t>European Journal of Political Economy</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>0176-2680</t>
@@ -28747,6 +29068,7 @@
           <t>European Journal of Pragmatism and American Philosophy</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>EJPAP</t>
@@ -28796,6 +29118,7 @@
       <c r="S143" t="n">
         <v>2009</v>
       </c>
+      <c r="T143" t="inlineStr"/>
       <c r="U143" t="inlineStr">
         <is>
           <t>2000's</t>
@@ -28809,6 +29132,7 @@
       <c r="W143" t="n">
         <v>2</v>
       </c>
+      <c r="X143" t="inlineStr"/>
       <c r="Y143" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -28946,6 +29270,7 @@
           <t>European Review of Applied Psychology</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>ERAP</t>
@@ -29093,16 +29418,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP144" t="inlineStr"/>
       <c r="AQ144" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR144" t="inlineStr"/>
       <c r="AS144" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT144" t="inlineStr"/>
       <c r="AU144" t="inlineStr">
         <is>
           <t>0</t>
@@ -29150,6 +29478,7 @@
           <t>Finance Contrôle Stratégie</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
           <t>FCS</t>
@@ -29204,6 +29533,7 @@
       <c r="S145" t="n">
         <v>1998</v>
       </c>
+      <c r="T145" t="inlineStr"/>
       <c r="U145" t="inlineStr">
         <is>
           <t>1990's</t>
@@ -29217,6 +29547,7 @@
       <c r="W145" t="n">
         <v>4</v>
       </c>
+      <c r="X145" t="inlineStr"/>
       <c r="Y145" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -29344,6 +29675,7 @@
           <t>First World War Studies</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>1947-5020</t>
@@ -29486,6 +29818,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -29844,16 +30177,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP148" t="inlineStr"/>
       <c r="AQ148" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR148" t="inlineStr"/>
       <c r="AS148" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT148" t="inlineStr"/>
       <c r="AU148" t="inlineStr">
         <is>
           <t>0</t>
@@ -29901,6 +30237,7 @@
           <t>Global Media and China</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>2059-4372</t>
@@ -30038,6 +30375,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -30060,6 +30398,7 @@
           <t>Histoire de l'art</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
           <t>0992-2059</t>
@@ -30202,11 +30541,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR150" t="inlineStr"/>
       <c r="AS150" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT150" t="inlineStr"/>
       <c r="AU150" t="inlineStr">
         <is>
           <t>0</t>
@@ -30460,6 +30801,7 @@
           <t>International Journal of Antennas and Propagation</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>1687-5869</t>
@@ -30599,16 +30941,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP152" t="inlineStr"/>
       <c r="AQ152" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR152" t="inlineStr"/>
       <c r="AS152" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT152" t="inlineStr"/>
       <c r="AU152" t="inlineStr">
         <is>
           <t>0</t>
@@ -30661,6 +31006,7 @@
           <t>International Journal of Economic Policy in Emerging Economies</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>1752-0452</t>
@@ -30803,6 +31149,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -30825,6 +31172,7 @@
           <t>International Journal of Electronic Trade</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>IJETrade</t>
@@ -30869,6 +31217,7 @@
       <c r="S154" t="n">
         <v>2023</v>
       </c>
+      <c r="T154" t="inlineStr"/>
       <c r="U154" t="inlineStr">
         <is>
           <t>2020's</t>
@@ -30882,6 +31231,7 @@
       <c r="W154" t="n">
         <v>4</v>
       </c>
+      <c r="X154" t="inlineStr"/>
       <c r="Y154" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -30972,6 +31322,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -30994,6 +31345,7 @@
           <t>International Journal of Sport Management and Marketing</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
           <t>1475-8962</t>
@@ -31136,6 +31488,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -31295,16 +31648,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP156" t="inlineStr"/>
       <c r="AQ156" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR156" t="inlineStr"/>
       <c r="AS156" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT156" t="inlineStr"/>
       <c r="AU156" t="inlineStr">
         <is>
           <t>0</t>
@@ -31352,6 +31708,7 @@
           <t>Journal for General Philosophy of Science</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
           <t>0925-4560</t>
@@ -31499,16 +31856,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP157" t="inlineStr"/>
       <c r="AQ157" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR157" t="inlineStr"/>
       <c r="AS157" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT157" t="inlineStr"/>
       <c r="AU157" t="inlineStr">
         <is>
           <t>0</t>
@@ -31556,6 +31916,7 @@
           <t>Journal of Applied Economics</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>1514-0326</t>
@@ -31698,6 +32059,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -31720,6 +32082,7 @@
           <t>Journal of Asset Management</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
           <t>1470-8272</t>
@@ -31852,16 +32215,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP159" t="inlineStr"/>
       <c r="AQ159" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR159" t="inlineStr"/>
       <c r="AS159" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT159" t="inlineStr"/>
       <c r="AU159" t="inlineStr">
         <is>
           <t>0</t>
@@ -31909,6 +32275,7 @@
           <t>Journal of Decision Systems</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
           <t>1246-0125</t>
@@ -32103,6 +32470,7 @@
           <t>Journal of Enterprise Information Management</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
           <t>1741-0398</t>
@@ -32240,16 +32608,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP161" t="inlineStr"/>
       <c r="AQ161" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR161" t="inlineStr"/>
       <c r="AS161" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT161" t="inlineStr"/>
       <c r="AU161" t="inlineStr">
         <is>
           <t>0</t>
@@ -32297,6 +32668,7 @@
           <t>Journal of Global History</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
           <t>1740-0228</t>
@@ -32429,16 +32801,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP162" t="inlineStr"/>
       <c r="AQ162" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR162" t="inlineStr"/>
       <c r="AS162" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT162" t="inlineStr"/>
       <c r="AU162" t="inlineStr">
         <is>
           <t>0</t>
@@ -32486,6 +32861,7 @@
           <t>Journal of Neurolinguistics</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
           <t>0911-6044</t>
@@ -32623,16 +32999,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP163" t="inlineStr"/>
       <c r="AQ163" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR163" t="inlineStr"/>
       <c r="AS163" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT163" t="inlineStr"/>
       <c r="AU163" t="inlineStr">
         <is>
           <t>0</t>
@@ -32680,6 +33059,7 @@
           <t>Journal of Urban Mobility</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
           <t>2667-0917</t>
@@ -32817,6 +33197,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -32981,16 +33362,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP165" t="inlineStr"/>
       <c r="AQ165" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR165" t="inlineStr"/>
       <c r="AS165" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT165" t="inlineStr"/>
       <c r="AU165" t="inlineStr">
         <is>
           <t>0</t>
@@ -33175,16 +33559,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP166" t="inlineStr"/>
       <c r="AQ166" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR166" t="inlineStr"/>
       <c r="AS166" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT166" t="inlineStr"/>
       <c r="AU166" t="inlineStr">
         <is>
           <t>0</t>
@@ -33232,6 +33619,7 @@
           <t>Latin American Antiquity</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
           <t>1045-6635</t>
@@ -33369,16 +33757,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP167" t="inlineStr"/>
       <c r="AQ167" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR167" t="inlineStr"/>
       <c r="AS167" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT167" t="inlineStr"/>
       <c r="AU167" t="inlineStr">
         <is>
           <t>0</t>
@@ -33595,6 +33986,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -33617,6 +34009,7 @@
           <t>Logistique et management</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>1250-7970</t>
@@ -33806,6 +34199,7 @@
           <t>Mechanics of Advanced Materials and Structures</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
           <t>1537-6494</t>
@@ -33948,6 +34342,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -34024,6 +34419,7 @@
       <c r="S171" t="n">
         <v>2024</v>
       </c>
+      <c r="T171" t="inlineStr"/>
       <c r="U171" t="inlineStr">
         <is>
           <t>2020's</t>
@@ -34037,6 +34433,7 @@
       <c r="W171" t="n">
         <v>2</v>
       </c>
+      <c r="X171" t="inlineStr"/>
       <c r="Y171" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -34137,6 +34534,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -34159,6 +34557,7 @@
           <t>Neuropsychiatrie de l'enfance et de l'adolescence</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
           <t>0222-9617</t>
@@ -34301,16 +34700,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP172" t="inlineStr"/>
       <c r="AQ172" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR172" t="inlineStr"/>
       <c r="AS172" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT172" t="inlineStr"/>
       <c r="AU172" t="inlineStr">
         <is>
           <t>0</t>
@@ -34505,6 +34907,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -34527,6 +34930,7 @@
           <t>Philosophies</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
           <t>2409-9287</t>
@@ -34723,6 +35127,7 @@
           <t>Political Anthropological Research on International Social Sciences</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>PARISS</t>
@@ -34767,6 +35172,7 @@
       <c r="S175" t="n">
         <v>2020</v>
       </c>
+      <c r="T175" t="inlineStr"/>
       <c r="U175" t="inlineStr">
         <is>
           <t>2020's</t>
@@ -34780,6 +35186,7 @@
       <c r="W175" t="n">
         <v>2</v>
       </c>
+      <c r="X175" t="inlineStr"/>
       <c r="Y175" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -34870,6 +35277,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -34892,6 +35300,7 @@
           <t>Revue des mondes musulmans et de la Méditerranée</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
           <t>REMMM</t>
@@ -34964,6 +35373,7 @@
       <c r="W176" t="n">
         <v>2</v>
       </c>
+      <c r="X176" t="inlineStr"/>
       <c r="Y176" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -35019,6 +35429,7 @@
           <t>CC BY-SA</t>
         </is>
       </c>
+      <c r="AL176" t="inlineStr"/>
       <c r="AM176" t="inlineStr">
         <is>
           <t>0</t>
@@ -35049,6 +35460,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AT176" t="inlineStr"/>
       <c r="AU176" t="inlineStr">
         <is>
           <t>1</t>
@@ -35106,6 +35518,7 @@
           <t>Requirements Engineering</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>0947-3602</t>
@@ -35238,16 +35651,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP177" t="inlineStr"/>
       <c r="AQ177" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR177" t="inlineStr"/>
       <c r="AS177" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT177" t="inlineStr"/>
       <c r="AU177" t="inlineStr">
         <is>
           <t>0</t>
@@ -35295,6 +35711,7 @@
           <t>Revue d'économie industrielle</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>0154-3229</t>
@@ -35412,6 +35829,7 @@
           <t>hybride</t>
         </is>
       </c>
+      <c r="AL178" t="inlineStr"/>
       <c r="AM178" t="inlineStr">
         <is>
           <t>0</t>
@@ -35494,6 +35912,7 @@
           <t>Revue d'histoire du théâtre</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>1291-2530</t>
@@ -35636,16 +36055,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP179" t="inlineStr"/>
       <c r="AQ179" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR179" t="inlineStr"/>
       <c r="AS179" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT179" t="inlineStr"/>
       <c r="AU179" t="inlineStr">
         <is>
           <t>0</t>
@@ -35693,6 +36115,7 @@
           <t>Revue des études byzantines</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>0766-5598</t>
@@ -35840,11 +36263,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AR180" t="inlineStr"/>
       <c r="AS180" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT180" t="inlineStr"/>
       <c r="AU180" t="inlineStr">
         <is>
           <t>0</t>
@@ -35892,6 +36317,7 @@
           <t>Revue interdisciplinaire d'études juridiques</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>RIEJ</t>
@@ -35946,6 +36372,7 @@
       <c r="S181" t="n">
         <v>1978</v>
       </c>
+      <c r="T181" t="inlineStr"/>
       <c r="U181" t="inlineStr">
         <is>
           <t>1970's</t>
@@ -36019,6 +36446,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL181" t="inlineStr"/>
       <c r="AM181" t="inlineStr">
         <is>
           <t>0</t>
@@ -36029,11 +36457,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP181" t="inlineStr"/>
       <c r="AQ181" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR181" t="inlineStr"/>
       <c r="AS181" t="inlineStr">
         <is>
           <t>1</t>
@@ -36091,6 +36521,7 @@
           <t>Revue internationale d'histoire militaire ancienne</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>HiMA</t>
@@ -36145,6 +36576,7 @@
       <c r="S182" t="n">
         <v>2015</v>
       </c>
+      <c r="T182" t="inlineStr"/>
       <c r="U182" t="inlineStr">
         <is>
           <t>2010's</t>
@@ -36158,6 +36590,7 @@
       <c r="W182" t="n">
         <v>1</v>
       </c>
+      <c r="X182" t="inlineStr"/>
       <c r="Y182" t="inlineStr">
         <is>
           <t>papier+numérique</t>
@@ -36228,16 +36661,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP182" t="inlineStr"/>
       <c r="AQ182" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR182" t="inlineStr"/>
       <c r="AS182" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT182" t="inlineStr"/>
       <c r="AU182" t="inlineStr">
         <is>
           <t>0</t>
@@ -36290,6 +36726,7 @@
           <t>Risk and Decision Analysis</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>1569-7371</t>
@@ -36432,6 +36869,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -36454,6 +36892,7 @@
           <t>Sahara et Sahel</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>2801-4472</t>
@@ -36611,6 +37050,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -36633,6 +37073,7 @@
           <t>Studies in Microeconomics</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>2321-0222</t>
@@ -36775,6 +37216,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -36797,6 +37239,7 @@
           <t>The European Journal of the History of Economic Thought</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>0967-2567</t>
@@ -36929,16 +37372,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP186" t="inlineStr"/>
       <c r="AQ186" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR186" t="inlineStr"/>
       <c r="AS186" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT186" t="inlineStr"/>
       <c r="AU186" t="inlineStr">
         <is>
           <t>0</t>
@@ -36986,6 +37432,7 @@
           <t>The Southern Journal of Philosophy</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>0038-4283</t>
@@ -37170,6 +37617,7 @@
           <t>The Spanish Journal of Psychology</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>1138-7416</t>
@@ -37359,6 +37807,7 @@
           <t>Théâtre/Public</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>0335-2927</t>
@@ -37543,6 +37992,7 @@
           <t>Theory and Decision</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>0040-5833</t>
@@ -37675,16 +38125,19 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP190" t="inlineStr"/>
       <c r="AQ190" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR190" t="inlineStr"/>
       <c r="AS190" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AT190" t="inlineStr"/>
       <c r="AU190" t="inlineStr">
         <is>
           <t>0</t>
@@ -37732,6 +38185,7 @@
           <t>Travail, genre et sociétés</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>1294-6303</t>
@@ -37854,6 +38308,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL191" t="inlineStr"/>
       <c r="AM191" t="inlineStr">
         <is>
           <t>0</t>
@@ -37864,11 +38319,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP191" t="inlineStr"/>
       <c r="AQ191" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR191" t="inlineStr"/>
       <c r="AS191" t="inlineStr">
         <is>
           <t>1</t>
@@ -37926,6 +38383,7 @@
           <t>Travaux et mémoires</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>0577-1471</t>
@@ -38249,6 +38707,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="BA193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -38393,6 +38852,7 @@
           <t>Tous droits réservés</t>
         </is>
       </c>
+      <c r="AL194" t="inlineStr"/>
       <c r="AM194" t="inlineStr">
         <is>
           <t>0</t>
@@ -38403,11 +38863,13 @@
           <t>0</t>
         </is>
       </c>
+      <c r="AP194" t="inlineStr"/>
       <c r="AQ194" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AR194" t="inlineStr"/>
       <c r="AS194" t="inlineStr">
         <is>
           <t>1</t>

</xml_diff>